<commit_message>
Add property dropdowns to business logs
Back both Property columns with a shared customizable list so time and mileage entries use consistent property names.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Business-Time-Mileage-Tracker.xlsx
+++ b/Business-Time-Mileage-Tracker.xlsx
@@ -1103,14 +1103,14 @@
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Customize activity choices</t>
+          <t>Customize dropdown choices</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Unhide the Lists sheet (Home &gt; Format &gt; Hide &amp; Unhide &gt; Unhide Sheet), edit the activity names, then hide it again. Keep the choices within cells A2:A11 so the dropdown continues to work.</t>
+          <t>Unhide the Lists sheet (Home &gt; Format &gt; Hide &amp; Unhide &gt; Unhide Sheet), edit activities in A2:A11 and properties in B2:B11, then hide it again. Keep choices within those ranges so the dropdowns continue to work.</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,10 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
+    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Select a listed property" error="Choose a property from the dropdown." promptTitle="Choose a property" prompt="Select a property or add one on the Lists sheet." type="list" errorStyle="stop">
+      <formula1>'Lists'!$B$2:$B$11</formula1>
+    </dataValidation>
     <dataValidation sqref="C2:C1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Select a listed activity" error="Choose an activity from the dropdown." promptTitle="Choose an activity" prompt="Select a common activity or add one on the Lists sheet." type="list" errorStyle="stop">
       <formula1>'Lists'!$A$2:$A$11</formula1>
     </dataValidation>
@@ -1779,7 +1782,10 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Select a listed property" error="Choose a property from the dropdown." promptTitle="Choose a property" prompt="Select a property or add one on the Lists sheet." type="list" errorStyle="stop">
+      <formula1>'Lists'!$B$2:$B$11</formula1>
+    </dataValidation>
     <dataValidation sqref="A2:A1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Invalid date" error="Enter a valid date between 2000 and 2100." promptTitle="Enter a date" prompt="Use a date between 2000 and 2100." type="date" errorStyle="stop" operator="between">
       <formula1>DATE(2000,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
@@ -1811,10 +1817,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1823,6 +1830,11 @@
           <t>Activity</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1830,6 +1842,11 @@
           <t>Administration</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Maple Street Duplex</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1837,6 +1854,11 @@
           <t>Bookkeeping</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Oak Avenue Rental</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1844,6 +1866,11 @@
           <t>Cleaning</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Property 3</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1851,6 +1878,11 @@
           <t>Inspections</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Property 4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1858,6 +1890,11 @@
           <t>Maintenance</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Property 5</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1865,6 +1902,11 @@
           <t>Marketing</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Property 6</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1872,6 +1914,11 @@
           <t>Property research</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Property 7</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1879,6 +1926,11 @@
           <t>Tenant communication</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Property 8</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1886,11 +1938,21 @@
           <t>Travel planning</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Property 9</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
           <t>Other</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Property 10</t>
         </is>
       </c>
     </row>

</xml_diff>